<commit_message>
Add tests for drift correction functionality and report parameters
- Implemented a test to verify drift tracking attributes in `test_drift.py`, ensuring the correct state before and after applying drift correction.
- Created a new test file `test_report_parameters.py` to validate the parameters sheet for drift information, checking both cases of drift correction applied and not applied.
</commit_message>
<xml_diff>
--- a/Water_18O_Report.xlsx
+++ b/Water_18O_Report.xlsx
@@ -1198,7 +1198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,20 +1291,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Slope</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1.053231857877764</v>
+          <t>Drift Correction Applied</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Drift Monitor Used</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Slope</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.053231857877764</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B12" t="n">
         <v>1.866694711662196</v>
       </c>
     </row>

</xml_diff>